<commit_message>
updated search products page scenarios and regression class
</commit_message>
<xml_diff>
--- a/ecommerse_mavne_project_setup_anjan_bharath_Shilpa_sharnya/project_documents.xlsx
+++ b/ecommerse_mavne_project_setup_anjan_bharath_Shilpa_sharnya/project_documents.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\eclipse_coding_projects\selenium_automation\ecommerse_mavne_project_setup_anjan_bharath_Shilpa_sharnya\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC0D7D91-5939-413E-9F42-1D6B077CDF98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{683F844E-ADD6-4416-93AC-FB3D6E76092E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-255" yWindow="16080" windowWidth="29040" windowHeight="16440" tabRatio="916" firstSheet="11" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="916" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Homepage" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="59">
   <si>
     <t>title</t>
   </si>
@@ -216,6 +216,24 @@
   </si>
   <si>
     <t>http://localhost:5173/single-product/&lt;id of the product&gt;</t>
+  </si>
+  <si>
+    <t>product names</t>
+  </si>
+  <si>
+    <t>apple</t>
+  </si>
+  <si>
+    <t>samsung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  yoga mat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pen    </t>
+  </si>
+  <si>
+    <t>water bottle</t>
   </si>
 </sst>
 </file>
@@ -1134,7 +1152,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3146659-BA30-470B-AE8C-F36F71E851DF}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.7109375" bestFit="1" customWidth="1"/>
@@ -1148,6 +1166,36 @@
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
brands section automation scripts
</commit_message>
<xml_diff>
--- a/ecommerse_mavne_project_setup_anjan_bharath_Shilpa_sharnya/project_documents.xlsx
+++ b/ecommerse_mavne_project_setup_anjan_bharath_Shilpa_sharnya/project_documents.xlsx
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="68">
   <si>
     <t>title</t>
   </si>
@@ -119,9 +119,6 @@
     <t>Contact Us | ECODERS</t>
   </si>
   <si>
-    <t>Elements in homepage</t>
-  </si>
-  <si>
     <t>Elements in footer section</t>
   </si>
   <si>
@@ -237,6 +234,27 @@
   </si>
   <si>
     <t>Showing 7 of 10 categories</t>
+  </si>
+  <si>
+    <t>All Brand Names</t>
+  </si>
+  <si>
+    <t>APPLE</t>
+  </si>
+  <si>
+    <t>SAMSUNG</t>
+  </si>
+  <si>
+    <t>SONY</t>
+  </si>
+  <si>
+    <t>Popular Brands</t>
+  </si>
+  <si>
+    <t>Smooth infinite marquee • drag / swipe anytime • tap to search</t>
+  </si>
+  <si>
+    <t>117 brands</t>
   </si>
 </sst>
 </file>
@@ -558,7 +576,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -566,18 +584,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.28515625" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" customWidth="1"/>
-    <col min="3" max="3" width="28.5703125" customWidth="1"/>
-    <col min="4" max="4" width="37" customWidth="1"/>
-    <col min="6" max="6" width="23" customWidth="1"/>
-    <col min="7" max="7" width="41.140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8">
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="42.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="58.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -585,7 +608,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -602,23 +625,47 @@
         <v>12345</v>
       </c>
       <c r="F2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G2" t="s">
         <v>59</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>60</v>
       </c>
-      <c r="H2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
+      <c r="I2" t="s">
+        <v>65</v>
+      </c>
+      <c r="J2" t="s">
+        <v>66</v>
+      </c>
+      <c r="K2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="D4" s="2">
         <v>49290</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
-      <c r="A6" t="s">
-        <v>22</v>
+    <row r="5" spans="1:11">
+      <c r="A5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -679,10 +726,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
         <v>25</v>
-      </c>
-      <c r="B2" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -709,10 +756,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="s">
         <v>27</v>
-      </c>
-      <c r="B2" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -739,10 +786,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" t="s">
         <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -769,11 +816,11 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B2" t="s">
         <v>35</v>
       </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -795,10 +842,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" t="s">
         <v>48</v>
+      </c>
+      <c r="B2" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -825,10 +872,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
         <v>29</v>
-      </c>
-      <c r="B2" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -855,10 +902,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" t="s">
         <v>31</v>
+      </c>
+      <c r="B2" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -885,10 +932,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" t="s">
         <v>37</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -915,11 +962,11 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
         <v>39</v>
       </c>
-      <c r="B2" t="s">
-        <v>40</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -936,7 +983,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -963,10 +1010,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
         <v>41</v>
-      </c>
-      <c r="B2" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -993,10 +1040,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" t="s">
         <v>43</v>
-      </c>
-      <c r="B2" t="s">
-        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1023,10 +1070,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B2" t="s">
-        <v>50</v>
+        <v>46</v>
+      </c>
+      <c r="B2" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1053,10 +1100,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1086,10 +1133,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" t="s">
         <v>45</v>
-      </c>
-      <c r="B2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1102,11 +1149,11 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" t="s">
         <v>45</v>
       </c>
-      <c r="B5" t="s">
-        <v>46</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1123,7 +1170,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1184,32 +1231,32 @@
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>